<commit_message>
fix unit for flux
</commit_message>
<xml_diff>
--- a/data/circular.xlsx
+++ b/data/circular.xlsx
@@ -1361,7 +1361,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SAO RAS</t>
+          <t>SAORAS</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>SAO RAS</t>
+          <t>SAORAS</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Osservatorio Astronomico "Nastro Verde"</t>
+          <t>OsservatorioAstronomicoNastroVerde</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Osservatorio Astronomico "Nastro Verde"</t>
+          <t>OsservatorioAstronomicoNastroVerde</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>SAO RAS</t>
+          <t>SAORAS</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Osservatorio Astronomico "Nastro Verde"</t>
+          <t>OsservatorioAstronomicoNastroVerde</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Osservatorio Astronomico "Nastro Verde"</t>
+          <t>OsservatorioAstronomicoNastroVerde</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Osservatorio Astronomico "Nastro Verde"</t>
+          <t>OsservatorioAstronomicoNastroVerde</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -3330,7 +3330,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Osservatorio Astronomico "Nastro Verde"</t>
+          <t>OsservatorioAstronomicoNastroVerde</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -3505,7 +3505,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3804,7 +3804,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -3936,7 +3936,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -4002,7 +4002,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Osservatorio Astronomico "Nastro Verde"</t>
+          <t>OsservatorioAstronomicoNastroVerde</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -4072,7 +4072,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Osservatorio Astronomico "Nastro Verde"</t>
+          <t>OsservatorioAstronomicoNastroVerde</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -4142,7 +4142,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -4177,7 +4177,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -4243,7 +4243,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -4278,7 +4278,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -4344,7 +4344,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -4513,7 +4513,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -4548,7 +4548,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4676,7 +4676,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -4746,7 +4746,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -4777,7 +4777,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -4882,7 +4882,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -4917,7 +4917,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -4952,7 +4952,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -5057,7 +5057,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -5197,7 +5197,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -5228,7 +5228,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -5263,7 +5263,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -5399,7 +5399,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -5465,7 +5465,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -5500,7 +5500,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -5601,7 +5601,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -5632,7 +5632,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -5733,7 +5733,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -5935,7 +5935,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -5970,7 +5970,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -6001,7 +6001,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -6063,7 +6063,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -6168,7 +6168,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -6265,7 +6265,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -6300,7 +6300,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -6366,7 +6366,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -6397,7 +6397,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -6432,7 +6432,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -6498,7 +6498,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -6529,7 +6529,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -6595,7 +6595,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASTER-SAAO </t>
+          <t>MASTER-SAAO</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -6700,7 +6700,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -6731,7 +6731,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -6766,7 +6766,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -6797,7 +6797,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -6832,7 +6832,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leavitt </t>
+          <t>Leavitt</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -6898,7 +6898,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -7003,7 +7003,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -7143,7 +7143,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -7213,7 +7213,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Bassano Bresciano Observatory</t>
+          <t>BassanoBrescianoObservatory</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -8547,7 +8547,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Liverpool Telescope</t>
+          <t>LiverpoolTelescope</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -8578,7 +8578,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Liverpool Telescope</t>
+          <t>LiverpoolTelescope</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -8609,7 +8609,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Liverpool Telescope</t>
+          <t>LiverpoolTelescope</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -8640,7 +8640,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Liverpool Telescope</t>
+          <t>LiverpoolTelescope</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Liverpool Telescope</t>
+          <t>LiverpoolTelescope</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -8737,7 +8737,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>SVOM/COLIBRÍ (FM-GFT)</t>
+          <t>SVOM/COLIBRÍ(FM-GFT)</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -8947,7 +8947,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t xml:space="preserve">SVOM/COLIBRÍ </t>
+          <t>SVOM/COLIBRÍ</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -8982,7 +8982,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t xml:space="preserve">SVOM/COLIBRÍ </t>
+          <t>SVOM/COLIBRÍ</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -9017,7 +9017,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t xml:space="preserve">SVOM/COLIBRÍ </t>
+          <t>SVOM/COLIBRÍ</t>
         </is>
       </c>
       <c r="D257" t="n">
@@ -9215,7 +9215,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t xml:space="preserve">JinShan </t>
+          <t>JinShan</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -9456,7 +9456,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>SAO RAS</t>
+          <t>SAORAS</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -9561,7 +9561,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>SAO RAS</t>
+          <t>SAORAS</t>
         </is>
       </c>
       <c r="D273" t="n">

</xml_diff>